<commit_message>
feat: rebuild UI with Tailwind design system, shared layouts and components
Introduces layouts/app and layouts/guest with a NavigationComposer, a
shared component library (card, table, page-header, status-badge, etc.),
and a compiled-locally Tailwind stylesheet across every screen. Keeps the
build fully offline-safe (no CDN or webfont fetches, system font stack,
inline data-URI icons) and documents the npm build step and physical
offline rehearsal check in CONTRIBUTING.md and deployment-rehearsal.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Gyx99g7Bsso5fz3Yb4HG2
</commit_message>
<xml_diff>
--- a/tests/Fixtures/register_clean.xlsx
+++ b/tests/Fixtures/register_clean.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramisys\municipal-payroll-system\tests\Fixtures\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A4C50EA-2753-4024-B112-926EF17A716E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Register" sheetId="1" r:id="rId4"/>
+    <sheet name="Register" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Employee No.</t>
   </si>
@@ -74,26 +79,21 @@
     <t>Net Pay</t>
   </si>
   <si>
-    <t>E-0001</t>
-  </si>
-  <si>
-    <t>E-0002</t>
-  </si>
-  <si>
-    <t>E-0003</t>
+    <t>E-1001</t>
+  </si>
+  <si>
+    <t>E-1002</t>
+  </si>
+  <si>
+    <t>E-1003</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -120,14 +120,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="2" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -417,14 +425,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S4"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -483,12 +488,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>19</v>
       </c>
       <c r="B2" s="1">
-        <v>20000.0</v>
+        <v>20000</v>
       </c>
       <c r="C2" s="1">
         <v>1500.5</v>
@@ -497,40 +502,40 @@
         <v>300.25</v>
       </c>
       <c r="E2" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F2" s="1">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="G2" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H2" s="1">
-        <v>900.0</v>
+        <v>900</v>
       </c>
       <c r="I2" s="1">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="J2" s="1">
-        <v>100.0</v>
+        <v>100</v>
       </c>
       <c r="K2" s="1">
-        <v>1200.35</v>
+        <v>1200.3499999999999</v>
       </c>
       <c r="L2" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="M2" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="N2" s="1">
-        <v>1800.0</v>
+        <v>1800</v>
       </c>
       <c r="O2" s="1">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="P2" s="1">
-        <v>100.0</v>
+        <v>100</v>
       </c>
       <c r="Q2" s="1">
         <v>23800.75</v>
@@ -539,60 +544,60 @@
         <v>2700.35</v>
       </c>
       <c r="S2" s="1">
-        <v>21100.4</v>
+        <v>21100.400000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:19">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>20</v>
       </c>
       <c r="B3" s="1">
-        <v>18000.0</v>
+        <v>18000</v>
       </c>
       <c r="C3" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="D3" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E3" s="1">
         <v>692.31</v>
       </c>
       <c r="F3" s="1">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="G3" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H3" s="1">
-        <v>810.0</v>
+        <v>810</v>
       </c>
       <c r="I3" s="1">
-        <v>450.0</v>
+        <v>450</v>
       </c>
       <c r="J3" s="1">
-        <v>100.0</v>
+        <v>100</v>
       </c>
       <c r="K3" s="1">
         <v>950.1</v>
       </c>
       <c r="L3" s="1">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="M3" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="N3" s="1">
-        <v>1620.0</v>
+        <v>1620</v>
       </c>
       <c r="O3" s="1">
-        <v>450.0</v>
+        <v>450</v>
       </c>
       <c r="P3" s="1">
-        <v>100.0</v>
+        <v>100</v>
       </c>
       <c r="Q3" s="1">
-        <v>20692.31</v>
+        <v>20692.310000000001</v>
       </c>
       <c r="R3" s="1">
         <v>2810.1</v>
@@ -601,54 +606,54 @@
         <v>17882.21</v>
       </c>
     </row>
-    <row r="4" spans="1:19">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
       <c r="B4" s="1">
-        <v>25000.0</v>
+        <v>25000</v>
       </c>
       <c r="C4" s="1">
         <v>2250.75</v>
       </c>
       <c r="D4" s="1">
-        <v>450.0</v>
+        <v>450</v>
       </c>
       <c r="E4" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F4" s="1">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="G4" s="1">
-        <v>25000.0</v>
+        <v>25000</v>
       </c>
       <c r="H4" s="1">
-        <v>1125.0</v>
+        <v>1125</v>
       </c>
       <c r="I4" s="1">
-        <v>625.0</v>
+        <v>625</v>
       </c>
       <c r="J4" s="1">
-        <v>100.0</v>
+        <v>100</v>
       </c>
       <c r="K4" s="1">
         <v>3200.55</v>
       </c>
       <c r="L4" s="1">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="M4" s="1">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="N4" s="1">
-        <v>2250.0</v>
+        <v>2250</v>
       </c>
       <c r="O4" s="1">
-        <v>625.0</v>
+        <v>625</v>
       </c>
       <c r="P4" s="1">
-        <v>100.0</v>
+        <v>100</v>
       </c>
       <c r="Q4" s="1">
         <v>54700.75</v>
@@ -661,8 +666,6 @@
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
 </file>
</xml_diff>